<commit_message>
Added New Zealand to equity_indices.xlsx
</commit_message>
<xml_diff>
--- a/data/equity_indices.xlsx
+++ b/data/equity_indices.xlsx
@@ -2,23 +2,25 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://uchicagoedu-my.sharepoint.com/personal/adiths_uchicago_edu/Documents/Classes/FINM 33150 Quantitative Trading Strategies/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="51" documentId="8_{22D9DAC2-4810-4A01-BDB3-CAF3552B4133}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{07DB9C32-7937-45F6-BD8B-6A1B327A6DC8}"/>
+  <xr:revisionPtr revIDLastSave="62" documentId="8_{22D9DAC2-4810-4A01-BDB3-CAF3552B4133}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{35DC6E44-9B7F-43D9-A0E0-05AF076F14ED}"/>
   <bookViews>
-    <workbookView xWindow="6315" yWindow="4815" windowWidth="28800" windowHeight="15345" xr2:uid="{3BCA3DED-04D9-4A67-87C5-E1AB33032BAA}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{3BCA3DED-04D9-4A67-87C5-E1AB33032BAA}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
     <definedName name="SpreadsheetBuilder_1" hidden="1">Sheet1!$A$1:$O$4</definedName>
+    <definedName name="SpreadsheetBuilder_2" hidden="1">Sheet2!$A$1:$B$7</definedName>
   </definedNames>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191028"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -39,7 +41,10 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="20">
+  <si>
+    <t>Dates</t>
+  </si>
   <si>
     <t>MEXBOL Index</t>
   </si>
@@ -83,7 +88,19 @@
     <t>JALSH Index</t>
   </si>
   <si>
-    <t>Dates</t>
+    <t>Start Date</t>
+  </si>
+  <si>
+    <t>End Date</t>
+  </si>
+  <si>
+    <t>NZ50SDE Index</t>
+  </si>
+  <si>
+    <t>PX_LAST</t>
+  </si>
+  <si>
+    <t>Last Price</t>
   </si>
 </sst>
 </file>
@@ -137,6 +154,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -456,57 +477,60 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DC25DC75-8F8C-40D9-AC00-9C3F98AC6D50}">
-  <dimension ref="A1:O1089"/>
+  <dimension ref="A1:P1089"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" t="s">
+        <v>11</v>
+      </c>
+      <c r="M1" t="s">
+        <v>12</v>
+      </c>
+      <c r="N1" t="s">
+        <v>13</v>
+      </c>
+      <c r="O1" t="s">
         <v>14</v>
       </c>
-      <c r="B1" t="s">
-        <v>0</v>
-      </c>
-      <c r="C1" t="s">
-        <v>1</v>
-      </c>
-      <c r="D1" t="s">
-        <v>2</v>
-      </c>
-      <c r="E1" t="s">
-        <v>3</v>
-      </c>
-      <c r="F1" t="s">
-        <v>4</v>
-      </c>
-      <c r="G1" t="s">
-        <v>5</v>
-      </c>
-      <c r="H1" t="s">
-        <v>6</v>
-      </c>
-      <c r="I1" t="s">
-        <v>7</v>
-      </c>
-      <c r="J1" t="s">
-        <v>8</v>
-      </c>
-      <c r="K1" t="s">
-        <v>9</v>
-      </c>
-      <c r="L1" t="s">
-        <v>10</v>
-      </c>
-      <c r="M1" t="s">
-        <v>11</v>
-      </c>
-      <c r="N1" t="s">
-        <v>12</v>
-      </c>
-      <c r="O1" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="2" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A2" s="1">
         <v>44564</v>
       </c>
@@ -552,8 +576,11 @@
       <c r="O2">
         <v>73722.600000000006</v>
       </c>
-    </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P2">
+        <v>2022.0219999999999</v>
+      </c>
+    </row>
+    <row r="3" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A3" s="1">
         <v>44565</v>
       </c>
@@ -599,8 +626,11 @@
       <c r="O3">
         <v>75052.06</v>
       </c>
-    </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P3">
+        <v>2022.0219999999999</v>
+      </c>
+    </row>
+    <row r="4" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A4" s="1">
         <v>44566</v>
       </c>
@@ -646,8 +676,11 @@
       <c r="O4">
         <v>75060.92</v>
       </c>
-    </row>
-    <row r="5" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P4">
+        <v>2022.0219999999999</v>
+      </c>
+    </row>
+    <row r="5" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A5" s="1">
         <v>44567</v>
       </c>
@@ -693,8 +726,11 @@
       <c r="O5">
         <v>74165.25</v>
       </c>
-    </row>
-    <row r="6" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P5">
+        <v>2022.0319999999999</v>
+      </c>
+    </row>
+    <row r="6" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A6" s="1">
         <v>44568</v>
       </c>
@@ -740,8 +776,11 @@
       <c r="O6">
         <v>73939.710000000006</v>
       </c>
-    </row>
-    <row r="7" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P6">
+        <v>2022.0319999999999</v>
+      </c>
+    </row>
+    <row r="7" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A7" s="1">
         <v>44571</v>
       </c>
@@ -787,8 +826,11 @@
       <c r="O7">
         <v>73830.47</v>
       </c>
-    </row>
-    <row r="8" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P7">
+        <v>2022.0319999999999</v>
+      </c>
+    </row>
+    <row r="8" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A8" s="1">
         <v>44572</v>
       </c>
@@ -834,8 +876,11 @@
       <c r="O8">
         <v>73971.429999999993</v>
       </c>
-    </row>
-    <row r="9" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P8">
+        <v>2022.0319999999999</v>
+      </c>
+    </row>
+    <row r="9" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A9" s="1">
         <v>44573</v>
       </c>
@@ -881,8 +926,11 @@
       <c r="O9">
         <v>75884.75</v>
       </c>
-    </row>
-    <row r="10" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P9">
+        <v>2022.0319999999999</v>
+      </c>
+    </row>
+    <row r="10" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A10" s="1">
         <v>44574</v>
       </c>
@@ -928,8 +976,11 @@
       <c r="O10">
         <v>75925.55</v>
       </c>
-    </row>
-    <row r="11" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P10">
+        <v>2022.0319999999999</v>
+      </c>
+    </row>
+    <row r="11" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A11" s="1">
         <v>44575</v>
       </c>
@@ -975,8 +1026,11 @@
       <c r="O11">
         <v>75160.210000000006</v>
       </c>
-    </row>
-    <row r="12" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P11">
+        <v>2022.0319999999999</v>
+      </c>
+    </row>
+    <row r="12" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A12" s="1">
         <v>44578</v>
       </c>
@@ -1022,8 +1076,11 @@
       <c r="O12">
         <v>75593.47</v>
       </c>
-    </row>
-    <row r="13" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P12">
+        <v>2022.0319999999999</v>
+      </c>
+    </row>
+    <row r="13" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A13" s="1">
         <v>44579</v>
       </c>
@@ -1069,8 +1126,11 @@
       <c r="O13">
         <v>74955.66</v>
       </c>
-    </row>
-    <row r="14" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P13">
+        <v>2022.0319999999999</v>
+      </c>
+    </row>
+    <row r="14" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A14" s="1">
         <v>44580</v>
       </c>
@@ -1116,8 +1176,11 @@
       <c r="O14">
         <v>76176.149999999994</v>
       </c>
-    </row>
-    <row r="15" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P14">
+        <v>2022.0319999999999</v>
+      </c>
+    </row>
+    <row r="15" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A15" s="1">
         <v>44581</v>
       </c>
@@ -1163,8 +1226,11 @@
       <c r="O15">
         <v>76233.259999999995</v>
       </c>
-    </row>
-    <row r="16" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P15">
+        <v>2022.0319999999999</v>
+      </c>
+    </row>
+    <row r="16" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A16" s="1">
         <v>44582</v>
       </c>
@@ -1210,8 +1276,11 @@
       <c r="O16">
         <v>74834.52</v>
       </c>
-    </row>
-    <row r="17" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P16">
+        <v>2022.0319999999999</v>
+      </c>
+    </row>
+    <row r="17" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A17" s="1">
         <v>44585</v>
       </c>
@@ -1257,8 +1326,11 @@
       <c r="O17">
         <v>72164.02</v>
       </c>
-    </row>
-    <row r="18" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P17">
+        <v>2022.0404000000001</v>
+      </c>
+    </row>
+    <row r="18" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A18" s="1">
         <v>44586</v>
       </c>
@@ -1304,8 +1376,11 @@
       <c r="O18">
         <v>72314.81</v>
       </c>
-    </row>
-    <row r="19" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P18">
+        <v>2022.04</v>
+      </c>
+    </row>
+    <row r="19" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A19" s="1">
         <v>44587</v>
       </c>
@@ -1351,8 +1426,11 @@
       <c r="O19">
         <v>73797.33</v>
       </c>
-    </row>
-    <row r="20" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P19">
+        <v>2022.04</v>
+      </c>
+    </row>
+    <row r="20" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A20" s="1">
         <v>44588</v>
       </c>
@@ -1398,8 +1476,11 @@
       <c r="O20">
         <v>73504.039999999994</v>
       </c>
-    </row>
-    <row r="21" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P20">
+        <v>2022.0429999999999</v>
+      </c>
+    </row>
+    <row r="21" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A21" s="1">
         <v>44589</v>
       </c>
@@ -1445,8 +1526,11 @@
       <c r="O21">
         <v>73454.960000000006</v>
       </c>
-    </row>
-    <row r="22" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P21">
+        <v>2022.0429999999999</v>
+      </c>
+    </row>
+    <row r="22" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A22" s="1">
         <v>44592</v>
       </c>
@@ -1492,8 +1576,11 @@
       <c r="O22">
         <v>74304.56</v>
       </c>
-    </row>
-    <row r="23" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P22">
+        <v>2022.05</v>
+      </c>
+    </row>
+    <row r="23" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A23" s="1">
         <v>44593</v>
       </c>
@@ -1539,8 +1626,11 @@
       <c r="O23">
         <v>74889.17</v>
       </c>
-    </row>
-    <row r="24" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P23">
+        <v>2022.05</v>
+      </c>
+    </row>
+    <row r="24" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A24" s="1">
         <v>44594</v>
       </c>
@@ -1586,8 +1676,11 @@
       <c r="O24">
         <v>75190.740000000005</v>
       </c>
-    </row>
-    <row r="25" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P24">
+        <v>2022.0501999999999</v>
+      </c>
+    </row>
+    <row r="25" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A25" s="1">
         <v>44595</v>
       </c>
@@ -1633,8 +1726,11 @@
       <c r="O25">
         <v>75021.67</v>
       </c>
-    </row>
-    <row r="26" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P25">
+        <v>2022.0619999999999</v>
+      </c>
+    </row>
+    <row r="26" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A26" s="1">
         <v>44596</v>
       </c>
@@ -1680,8 +1776,11 @@
       <c r="O26">
         <v>75206</v>
       </c>
-    </row>
-    <row r="27" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P26">
+        <v>2022.0619999999999</v>
+      </c>
+    </row>
+    <row r="27" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A27" s="1">
         <v>44599</v>
       </c>
@@ -1727,8 +1826,11 @@
       <c r="O27">
         <v>75679.56</v>
       </c>
-    </row>
-    <row r="28" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P27">
+        <v>2022.0619999999999</v>
+      </c>
+    </row>
+    <row r="28" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A28" s="1">
         <v>44600</v>
       </c>
@@ -1774,8 +1876,11 @@
       <c r="O28">
         <v>76090.52</v>
       </c>
-    </row>
-    <row r="29" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P28">
+        <v>2022.0619999999999</v>
+      </c>
+    </row>
+    <row r="29" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A29" s="1">
         <v>44601</v>
       </c>
@@ -1821,8 +1926,11 @@
       <c r="O29">
         <v>76690.92</v>
       </c>
-    </row>
-    <row r="30" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P29">
+        <v>2022.0619999999999</v>
+      </c>
+    </row>
+    <row r="30" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A30" s="1">
         <v>44602</v>
       </c>
@@ -1868,8 +1976,11 @@
       <c r="O30">
         <v>76585.19</v>
       </c>
-    </row>
-    <row r="31" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P30">
+        <v>2022.0619999999999</v>
+      </c>
+    </row>
+    <row r="31" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A31" s="1">
         <v>44603</v>
       </c>
@@ -1915,8 +2026,11 @@
       <c r="O31">
         <v>76382.95</v>
       </c>
-    </row>
-    <row r="32" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P31">
+        <v>2022.0619999999999</v>
+      </c>
+    </row>
+    <row r="32" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A32" s="1">
         <v>44606</v>
       </c>
@@ -1962,8 +2076,11 @@
       <c r="O32">
         <v>75765.16</v>
       </c>
-    </row>
-    <row r="33" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P32">
+        <v>2022.0619999999999</v>
+      </c>
+    </row>
+    <row r="33" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A33" s="1">
         <v>44607</v>
       </c>
@@ -2009,8 +2126,11 @@
       <c r="O33">
         <v>75853.16</v>
       </c>
-    </row>
-    <row r="34" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P33">
+        <v>2022.0619999999999</v>
+      </c>
+    </row>
+    <row r="34" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A34" s="1">
         <v>44608</v>
       </c>
@@ -2056,8 +2176,11 @@
       <c r="O34">
         <v>76502.59</v>
       </c>
-    </row>
-    <row r="35" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P34">
+        <v>2022.0619999999999</v>
+      </c>
+    </row>
+    <row r="35" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A35" s="1">
         <v>44609</v>
       </c>
@@ -2103,8 +2226,11 @@
       <c r="O35">
         <v>76154.69</v>
       </c>
-    </row>
-    <row r="36" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P35">
+        <v>2022.0619999999999</v>
+      </c>
+    </row>
+    <row r="36" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A36" s="1">
         <v>44610</v>
       </c>
@@ -2150,8 +2276,11 @@
       <c r="O36">
         <v>76368.34</v>
       </c>
-    </row>
-    <row r="37" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P36">
+        <v>2022.0721000000001</v>
+      </c>
+    </row>
+    <row r="37" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A37" s="1">
         <v>44613</v>
       </c>
@@ -2197,8 +2326,11 @@
       <c r="O37">
         <v>75528.460000000006</v>
       </c>
-    </row>
-    <row r="38" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P37">
+        <v>2022.0719999999999</v>
+      </c>
+    </row>
+    <row r="38" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A38" s="1">
         <v>44614</v>
       </c>
@@ -2244,8 +2376,11 @@
       <c r="O38">
         <v>75653.84</v>
       </c>
-    </row>
-    <row r="39" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P38">
+        <v>2022.0719999999999</v>
+      </c>
+    </row>
+    <row r="39" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A39" s="1">
         <v>44615</v>
       </c>
@@ -2291,8 +2426,11 @@
       <c r="O39">
         <v>74987.05</v>
       </c>
-    </row>
-    <row r="40" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P39">
+        <v>2022.0920000000001</v>
+      </c>
+    </row>
+    <row r="40" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A40" s="1">
         <v>44616</v>
       </c>
@@ -2338,8 +2476,11 @@
       <c r="O40">
         <v>73697.11</v>
       </c>
-    </row>
-    <row r="41" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P40">
+        <v>2022.0920000000001</v>
+      </c>
+    </row>
+    <row r="41" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A41" s="1">
         <v>44617</v>
       </c>
@@ -2385,8 +2526,11 @@
       <c r="O41">
         <v>74205.69</v>
       </c>
-    </row>
-    <row r="42" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P41">
+        <v>2022.0920000000001</v>
+      </c>
+    </row>
+    <row r="42" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A42" s="1">
         <v>44620</v>
       </c>
@@ -2432,8 +2576,11 @@
       <c r="O42">
         <v>76090.509999999995</v>
       </c>
-    </row>
-    <row r="43" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P42">
+        <v>2022.0920000000001</v>
+      </c>
+    </row>
+    <row r="43" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A43" s="1">
         <v>44621</v>
       </c>
@@ -2479,8 +2626,11 @@
       <c r="O43">
         <v>77110.69</v>
       </c>
-    </row>
-    <row r="44" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P43">
+        <v>2022.0920000000001</v>
+      </c>
+    </row>
+    <row r="44" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A44" s="1">
         <v>44622</v>
       </c>
@@ -2526,8 +2676,11 @@
       <c r="O44">
         <v>77536.12</v>
       </c>
-    </row>
-    <row r="45" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P44">
+        <v>2022.0920000000001</v>
+      </c>
+    </row>
+    <row r="45" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A45" s="1">
         <v>44623</v>
       </c>
@@ -2573,8 +2726,11 @@
       <c r="O45">
         <v>77390.850000000006</v>
       </c>
-    </row>
-    <row r="46" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P45">
+        <v>2022.0920000000001</v>
+      </c>
+    </row>
+    <row r="46" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A46" s="1">
         <v>44624</v>
       </c>
@@ -2620,8 +2776,11 @@
       <c r="O46">
         <v>74734.37</v>
       </c>
-    </row>
-    <row r="47" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P46">
+        <v>2022.0920000000001</v>
+      </c>
+    </row>
+    <row r="47" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A47" s="1">
         <v>44627</v>
       </c>
@@ -2667,8 +2826,11 @@
       <c r="O47">
         <v>73295.88</v>
       </c>
-    </row>
-    <row r="48" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P47">
+        <v>2022.0920000000001</v>
+      </c>
+    </row>
+    <row r="48" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A48" s="1">
         <v>44628</v>
       </c>
@@ -2714,8 +2876,11 @@
       <c r="O48">
         <v>72398.62</v>
       </c>
-    </row>
-    <row r="49" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P48">
+        <v>2022.0920000000001</v>
+      </c>
+    </row>
+    <row r="49" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A49" s="1">
         <v>44629</v>
       </c>
@@ -2761,8 +2926,11 @@
       <c r="O49">
         <v>72684.820000000007</v>
       </c>
-    </row>
-    <row r="50" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P49">
+        <v>2022.0920000000001</v>
+      </c>
+    </row>
+    <row r="50" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A50" s="1">
         <v>44630</v>
       </c>
@@ -2808,8 +2976,11 @@
       <c r="O50">
         <v>73889.41</v>
       </c>
-    </row>
-    <row r="51" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P50">
+        <v>2022.0920000000001</v>
+      </c>
+    </row>
+    <row r="51" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A51" s="1">
         <v>44631</v>
       </c>
@@ -2855,8 +3026,11 @@
       <c r="O51">
         <v>73685.89</v>
       </c>
-    </row>
-    <row r="52" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P51">
+        <v>2022.0930000000001</v>
+      </c>
+    </row>
+    <row r="52" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A52" s="1">
         <v>44634</v>
       </c>
@@ -2902,8 +3076,11 @@
       <c r="O52">
         <v>71903.72</v>
       </c>
-    </row>
-    <row r="53" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P52">
+        <v>2022.0930000000001</v>
+      </c>
+    </row>
+    <row r="53" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A53" s="1">
         <v>44635</v>
       </c>
@@ -2949,8 +3126,11 @@
       <c r="O53">
         <v>70628.2</v>
       </c>
-    </row>
-    <row r="54" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P53">
+        <v>2022.0930000000001</v>
+      </c>
+    </row>
+    <row r="54" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A54" s="1">
         <v>44636</v>
       </c>
@@ -2996,8 +3176,11 @@
       <c r="O54">
         <v>73484.3</v>
       </c>
-    </row>
-    <row r="55" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P54">
+        <v>2022.0930000000001</v>
+      </c>
+    </row>
+    <row r="55" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A55" s="1">
         <v>44637</v>
       </c>
@@ -3043,8 +3226,11 @@
       <c r="O55">
         <v>74124.27</v>
       </c>
-    </row>
-    <row r="56" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P55">
+        <v>2022.0930000000001</v>
+      </c>
+    </row>
+    <row r="56" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A56" s="1">
         <v>44638</v>
       </c>
@@ -3090,8 +3276,11 @@
       <c r="O56">
         <v>74847.63</v>
       </c>
-    </row>
-    <row r="57" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P56">
+        <v>2022.1122</v>
+      </c>
+    </row>
+    <row r="57" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A57" s="1">
         <v>44641</v>
       </c>
@@ -3137,8 +3326,11 @@
       <c r="O57">
         <v>74847.63</v>
       </c>
-    </row>
-    <row r="58" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P57">
+        <v>2022.1120000000001</v>
+      </c>
+    </row>
+    <row r="58" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A58" s="1">
         <v>44642</v>
       </c>
@@ -3184,8 +3376,11 @@
       <c r="O58">
         <v>75751.41</v>
       </c>
-    </row>
-    <row r="59" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P58">
+        <v>2022.1120000000001</v>
+      </c>
+    </row>
+    <row r="59" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A59" s="1">
         <v>44643</v>
       </c>
@@ -3231,8 +3426,11 @@
       <c r="O59">
         <v>74838.09</v>
       </c>
-    </row>
-    <row r="60" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P59">
+        <v>2022.1122</v>
+      </c>
+    </row>
+    <row r="60" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A60" s="1">
         <v>44644</v>
       </c>
@@ -3278,8 +3476,11 @@
       <c r="O60">
         <v>74349.94</v>
       </c>
-    </row>
-    <row r="61" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P60">
+        <v>2022.1122</v>
+      </c>
+    </row>
+    <row r="61" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A61" s="1">
         <v>44645</v>
       </c>
@@ -3325,8 +3526,11 @@
       <c r="O61">
         <v>74324.67</v>
       </c>
-    </row>
-    <row r="62" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P61">
+        <v>2022.1120000000001</v>
+      </c>
+    </row>
+    <row r="62" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A62" s="1">
         <v>44648</v>
       </c>
@@ -3372,8 +3576,11 @@
       <c r="O62">
         <v>74194.350000000006</v>
       </c>
-    </row>
-    <row r="63" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P62">
+        <v>2022.1120000000001</v>
+      </c>
+    </row>
+    <row r="63" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A63" s="1">
         <v>44649</v>
       </c>
@@ -3419,8 +3626,11 @@
       <c r="O63">
         <v>74776.39</v>
       </c>
-    </row>
-    <row r="64" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P63">
+        <v>2022.1120000000001</v>
+      </c>
+    </row>
+    <row r="64" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A64" s="1">
         <v>44650</v>
       </c>
@@ -3466,8 +3676,11 @@
       <c r="O64">
         <v>75425.31</v>
       </c>
-    </row>
-    <row r="65" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P64">
+        <v>2022.1220000000001</v>
+      </c>
+    </row>
+    <row r="65" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A65" s="1">
         <v>44651</v>
       </c>
@@ -3513,8 +3726,11 @@
       <c r="O65">
         <v>75497.149999999994</v>
       </c>
-    </row>
-    <row r="66" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P65">
+        <v>2022.1220000000001</v>
+      </c>
+    </row>
+    <row r="66" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A66" s="1">
         <v>44652</v>
       </c>
@@ -3560,8 +3776,11 @@
       <c r="O66">
         <v>75907.899999999994</v>
       </c>
-    </row>
-    <row r="67" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P66">
+        <v>2022.1220000000001</v>
+      </c>
+    </row>
+    <row r="67" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A67" s="1">
         <v>44655</v>
       </c>
@@ -3607,8 +3826,11 @@
       <c r="O67">
         <v>75835.070000000007</v>
       </c>
-    </row>
-    <row r="68" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P67">
+        <v>2022.1220000000001</v>
+      </c>
+    </row>
+    <row r="68" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A68" s="1">
         <v>44656</v>
       </c>
@@ -3654,8 +3876,11 @@
       <c r="O68">
         <v>75286.61</v>
       </c>
-    </row>
-    <row r="69" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P68">
+        <v>2022.1220000000001</v>
+      </c>
+    </row>
+    <row r="69" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A69" s="1">
         <v>44657</v>
       </c>
@@ -3701,8 +3926,11 @@
       <c r="O69">
         <v>74359.03</v>
       </c>
-    </row>
-    <row r="70" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P69">
+        <v>2022.1220000000001</v>
+      </c>
+    </row>
+    <row r="70" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A70" s="1">
         <v>44658</v>
       </c>
@@ -3748,8 +3976,11 @@
       <c r="O70">
         <v>74008.070000000007</v>
       </c>
-    </row>
-    <row r="71" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P70">
+        <v>2022.1220000000001</v>
+      </c>
+    </row>
+    <row r="71" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A71" s="1">
         <v>44659</v>
       </c>
@@ -3795,8 +4026,11 @@
       <c r="O71">
         <v>74776.11</v>
       </c>
-    </row>
-    <row r="72" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P71">
+        <v>2022.1220000000001</v>
+      </c>
+    </row>
+    <row r="72" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A72" s="1">
         <v>44662</v>
       </c>
@@ -3842,8 +4076,11 @@
       <c r="O72">
         <v>74426.399999999994</v>
       </c>
-    </row>
-    <row r="73" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P72">
+        <v>2022.1220000000001</v>
+      </c>
+    </row>
+    <row r="73" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A73" s="1">
         <v>44663</v>
       </c>
@@ -3889,8 +4126,11 @@
       <c r="O73">
         <v>73801.88</v>
       </c>
-    </row>
-    <row r="74" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P73">
+        <v>2022.1219000000001</v>
+      </c>
+    </row>
+    <row r="74" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A74" s="1">
         <v>44664</v>
       </c>
@@ -3936,8 +4176,11 @@
       <c r="O74">
         <v>73128.649999999994</v>
       </c>
-    </row>
-    <row r="75" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P74">
+        <v>2022.1220000000001</v>
+      </c>
+    </row>
+    <row r="75" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A75" s="1">
         <v>44665</v>
       </c>
@@ -3983,8 +4226,11 @@
       <c r="O75">
         <v>73382.83</v>
       </c>
-    </row>
-    <row r="76" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P75">
+        <v>2022.1220000000001</v>
+      </c>
+    </row>
+    <row r="76" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A76" s="1">
         <v>44666</v>
       </c>
@@ -4030,8 +4276,11 @@
       <c r="O76">
         <v>73382.83</v>
       </c>
-    </row>
-    <row r="77" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P76">
+        <v>2023.0219999999999</v>
+      </c>
+    </row>
+    <row r="77" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A77" s="1">
         <v>44669</v>
       </c>
@@ -4077,8 +4326,11 @@
       <c r="O77">
         <v>73382.83</v>
       </c>
-    </row>
-    <row r="78" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P77">
+        <v>2023.0219999999999</v>
+      </c>
+    </row>
+    <row r="78" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A78" s="1">
         <v>44670</v>
       </c>
@@ -4124,8 +4376,11 @@
       <c r="O78">
         <v>73830.27</v>
       </c>
-    </row>
-    <row r="79" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P78">
+        <v>2023.0219999999999</v>
+      </c>
+    </row>
+    <row r="79" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A79" s="1">
         <v>44671</v>
       </c>
@@ -4171,8 +4426,11 @@
       <c r="O79">
         <v>73783.429999999993</v>
       </c>
-    </row>
-    <row r="80" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P79">
+        <v>2023.0219999999999</v>
+      </c>
+    </row>
+    <row r="80" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A80" s="1">
         <v>44672</v>
       </c>
@@ -4218,8 +4476,11 @@
       <c r="O80">
         <v>73350.94</v>
       </c>
-    </row>
-    <row r="81" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P80">
+        <v>2023.0319999999999</v>
+      </c>
+    </row>
+    <row r="81" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A81" s="1">
         <v>44673</v>
       </c>
@@ -4265,8 +4526,11 @@
       <c r="O81">
         <v>72264.899999999994</v>
       </c>
-    </row>
-    <row r="82" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P81">
+        <v>2023.0319999999999</v>
+      </c>
+    </row>
+    <row r="82" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A82" s="1">
         <v>44676</v>
       </c>
@@ -4312,8 +4576,11 @@
       <c r="O82">
         <v>69750.67</v>
       </c>
-    </row>
-    <row r="83" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P82">
+        <v>2023.0319999999999</v>
+      </c>
+    </row>
+    <row r="83" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A83" s="1">
         <v>44677</v>
       </c>
@@ -4359,8 +4626,11 @@
       <c r="O83">
         <v>70264.11</v>
       </c>
-    </row>
-    <row r="84" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P83">
+        <v>2023.0319999999999</v>
+      </c>
+    </row>
+    <row r="84" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A84" s="1">
         <v>44678</v>
       </c>
@@ -4406,8 +4676,11 @@
       <c r="O84">
         <v>70264.11</v>
       </c>
-    </row>
-    <row r="85" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P84">
+        <v>2023.0319999999999</v>
+      </c>
+    </row>
+    <row r="85" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A85" s="1">
         <v>44679</v>
       </c>
@@ -4453,8 +4726,11 @@
       <c r="O85">
         <v>71534.570000000007</v>
       </c>
-    </row>
-    <row r="86" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P85">
+        <v>2023.0319999999999</v>
+      </c>
+    </row>
+    <row r="86" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A86" s="1">
         <v>44680</v>
       </c>
@@ -4500,8 +4776,11 @@
       <c r="O86">
         <v>72438.25</v>
       </c>
-    </row>
-    <row r="87" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P86">
+        <v>2023.0319999999999</v>
+      </c>
+    </row>
+    <row r="87" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A87" s="1">
         <v>44683</v>
       </c>
@@ -4547,8 +4826,11 @@
       <c r="O87">
         <v>72438.25</v>
       </c>
-    </row>
-    <row r="88" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P87">
+        <v>2023.0319999999999</v>
+      </c>
+    </row>
+    <row r="88" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A88" s="1">
         <v>44684</v>
       </c>
@@ -4594,8 +4876,11 @@
       <c r="O88">
         <v>71338.990000000005</v>
       </c>
-    </row>
-    <row r="89" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P88">
+        <v>2023.0319999999999</v>
+      </c>
+    </row>
+    <row r="89" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A89" s="1">
         <v>44685</v>
       </c>
@@ -4641,8 +4926,11 @@
       <c r="O89">
         <v>70357.58</v>
       </c>
-    </row>
-    <row r="90" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P89">
+        <v>2023.0319999999999</v>
+      </c>
+    </row>
+    <row r="90" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A90" s="1">
         <v>44686</v>
       </c>
@@ -4688,8 +4976,11 @@
       <c r="O90">
         <v>69682.649999999994</v>
       </c>
-    </row>
-    <row r="91" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P90">
+        <v>2023.0219999999999</v>
+      </c>
+    </row>
+    <row r="91" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A91" s="1">
         <v>44687</v>
       </c>
@@ -4735,8 +5026,11 @@
       <c r="O91">
         <v>67978.14</v>
       </c>
-    </row>
-    <row r="92" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P91">
+        <v>2023.0319999999999</v>
+      </c>
+    </row>
+    <row r="92" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A92" s="1">
         <v>44690</v>
       </c>
@@ -4782,8 +5076,11 @@
       <c r="O92">
         <v>66769.119999999995</v>
       </c>
-    </row>
-    <row r="93" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P92">
+        <v>2023.0509999999999</v>
+      </c>
+    </row>
+    <row r="93" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A93" s="1">
         <v>44691</v>
       </c>
@@ -4829,8 +5126,11 @@
       <c r="O93">
         <v>66966.73</v>
       </c>
-    </row>
-    <row r="94" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P93">
+        <v>2023.0509999999999</v>
+      </c>
+    </row>
+    <row r="94" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A94" s="1">
         <v>44692</v>
       </c>
@@ -4876,8 +5176,11 @@
       <c r="O94">
         <v>68416.41</v>
       </c>
-    </row>
-    <row r="95" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P94">
+        <v>2023.0509999999999</v>
+      </c>
+    </row>
+    <row r="95" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A95" s="1">
         <v>44693</v>
       </c>
@@ -4923,8 +5226,11 @@
       <c r="O95">
         <v>67251.89</v>
       </c>
-    </row>
-    <row r="96" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P95">
+        <v>2023.0509999999999</v>
+      </c>
+    </row>
+    <row r="96" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A96" s="1">
         <v>44694</v>
       </c>
@@ -4970,8 +5276,11 @@
       <c r="O96">
         <v>68650.66</v>
       </c>
-    </row>
-    <row r="97" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P96">
+        <v>2023.0509999999999</v>
+      </c>
+    </row>
+    <row r="97" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A97" s="1">
         <v>44697</v>
       </c>
@@ -5017,8 +5326,11 @@
       <c r="O97">
         <v>69211.759999999995</v>
       </c>
-    </row>
-    <row r="98" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P97">
+        <v>2023.0509999999999</v>
+      </c>
+    </row>
+    <row r="98" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A98" s="1">
         <v>44698</v>
       </c>
@@ -5064,8 +5376,11 @@
       <c r="O98">
         <v>69696.39</v>
       </c>
-    </row>
-    <row r="99" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P98">
+        <v>2023.0509999999999</v>
+      </c>
+    </row>
+    <row r="99" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A99" s="1">
         <v>44699</v>
       </c>
@@ -5111,8 +5426,11 @@
       <c r="O99">
         <v>69083.44</v>
       </c>
-    </row>
-    <row r="100" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P99">
+        <v>2023.0619999999999</v>
+      </c>
+    </row>
+    <row r="100" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A100" s="1">
         <v>44700</v>
       </c>
@@ -5158,8 +5476,11 @@
       <c r="O100">
         <v>68245.84</v>
       </c>
-    </row>
-    <row r="101" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P100">
+        <v>2023.0619999999999</v>
+      </c>
+    </row>
+    <row r="101" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A101" s="1">
         <v>44701</v>
       </c>
@@ -5205,8 +5526,11 @@
       <c r="O101">
         <v>67575.28</v>
       </c>
-    </row>
-    <row r="102" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P101">
+        <v>2023.0619999999999</v>
+      </c>
+    </row>
+    <row r="102" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A102" s="1">
         <v>44704</v>
       </c>
@@ -5252,8 +5576,11 @@
       <c r="O102">
         <v>68367.37</v>
       </c>
-    </row>
-    <row r="103" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P102">
+        <v>2023.0619999999999</v>
+      </c>
+    </row>
+    <row r="103" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A103" s="1">
         <v>44705</v>
       </c>
@@ -5299,8 +5626,11 @@
       <c r="O103">
         <v>67690.720000000001</v>
       </c>
-    </row>
-    <row r="104" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P103">
+        <v>2023.0619999999999</v>
+      </c>
+    </row>
+    <row r="104" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A104" s="1">
         <v>44706</v>
       </c>
@@ -5346,8 +5676,11 @@
       <c r="O104">
         <v>67585.25</v>
       </c>
-    </row>
-    <row r="105" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P104">
+        <v>2023.0619999999999</v>
+      </c>
+    </row>
+    <row r="105" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A105" s="1">
         <v>44707</v>
       </c>
@@ -5393,8 +5726,11 @@
       <c r="O105">
         <v>69483.759999999995</v>
       </c>
-    </row>
-    <row r="106" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P105">
+        <v>2023.0619999999999</v>
+      </c>
+    </row>
+    <row r="106" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A106" s="1">
         <v>44708</v>
       </c>
@@ -5440,8 +5776,11 @@
       <c r="O106">
         <v>70485.460000000006</v>
       </c>
-    </row>
-    <row r="107" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P106">
+        <v>2023.0619999999999</v>
+      </c>
+    </row>
+    <row r="107" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A107" s="1">
         <v>44711</v>
       </c>
@@ -5487,8 +5826,11 @@
       <c r="O107">
         <v>71958.149999999994</v>
       </c>
-    </row>
-    <row r="108" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P107">
+        <v>2023.0619999999999</v>
+      </c>
+    </row>
+    <row r="108" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A108" s="1">
         <v>44712</v>
       </c>
@@ -5534,8 +5876,11 @@
       <c r="O108">
         <v>72094.87</v>
       </c>
-    </row>
-    <row r="109" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P108">
+        <v>2023.0619999999999</v>
+      </c>
+    </row>
+    <row r="109" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A109" s="1">
         <v>44713</v>
       </c>
@@ -5581,8 +5926,11 @@
       <c r="O109">
         <v>70849.38</v>
       </c>
-    </row>
-    <row r="110" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P109">
+        <v>2023.0626</v>
+      </c>
+    </row>
+    <row r="110" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A110" s="1">
         <v>44714</v>
       </c>
@@ -5628,8 +5976,11 @@
       <c r="O110">
         <v>71035</v>
       </c>
-    </row>
-    <row r="111" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P110">
+        <v>2023.0626</v>
+      </c>
+    </row>
+    <row r="111" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A111" s="1">
         <v>44715</v>
       </c>
@@ -5675,8 +6026,11 @@
       <c r="O111">
         <v>70920.45</v>
       </c>
-    </row>
-    <row r="112" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P111">
+        <v>2023.0630000000001</v>
+      </c>
+    </row>
+    <row r="112" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A112" s="1">
         <v>44718</v>
       </c>
@@ -5722,8 +6076,11 @@
       <c r="O112">
         <v>71120.09</v>
       </c>
-    </row>
-    <row r="113" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P112">
+        <v>2023.0630000000001</v>
+      </c>
+    </row>
+    <row r="113" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A113" s="1">
         <v>44719</v>
       </c>
@@ -5769,8 +6126,11 @@
       <c r="O113">
         <v>70318.23</v>
       </c>
-    </row>
-    <row r="114" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P113">
+        <v>2023.0630000000001</v>
+      </c>
+    </row>
+    <row r="114" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A114" s="1">
         <v>44720</v>
       </c>
@@ -5816,8 +6176,11 @@
       <c r="O114">
         <v>69950.210000000006</v>
       </c>
-    </row>
-    <row r="115" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P114">
+        <v>2023.0630000000001</v>
+      </c>
+    </row>
+    <row r="115" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A115" s="1">
         <v>44721</v>
       </c>
@@ -5863,8 +6226,11 @@
       <c r="O115">
         <v>68910.8</v>
       </c>
-    </row>
-    <row r="116" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P115">
+        <v>2023.0709999999999</v>
+      </c>
+    </row>
+    <row r="116" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A116" s="1">
         <v>44722</v>
       </c>
@@ -5910,8 +6276,11 @@
       <c r="O116">
         <v>67803.509999999995</v>
       </c>
-    </row>
-    <row r="117" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P116">
+        <v>2023.0920000000001</v>
+      </c>
+    </row>
+    <row r="117" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A117" s="1">
         <v>44725</v>
       </c>
@@ -5957,8 +6326,11 @@
       <c r="O117">
         <v>66381.03</v>
       </c>
-    </row>
-    <row r="118" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P117">
+        <v>2023.0920000000001</v>
+      </c>
+    </row>
+    <row r="118" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A118" s="1">
         <v>44726</v>
       </c>
@@ -6004,8 +6376,11 @@
       <c r="O118">
         <v>65683.520000000004</v>
       </c>
-    </row>
-    <row r="119" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P118">
+        <v>2023.0920000000001</v>
+      </c>
+    </row>
+    <row r="119" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A119" s="1">
         <v>44727</v>
       </c>
@@ -6051,8 +6426,11 @@
       <c r="O119">
         <v>67502.09</v>
       </c>
-    </row>
-    <row r="120" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P119">
+        <v>2023.0920000000001</v>
+      </c>
+    </row>
+    <row r="120" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A120" s="1">
         <v>44728</v>
       </c>
@@ -6098,8 +6476,11 @@
       <c r="O120">
         <v>67502.09</v>
       </c>
-    </row>
-    <row r="121" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P120">
+        <v>2023.0920000000001</v>
+      </c>
+    </row>
+    <row r="121" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A121" s="1">
         <v>44729</v>
       </c>
@@ -6145,8 +6526,11 @@
       <c r="O121">
         <v>65390.879999999997</v>
       </c>
-    </row>
-    <row r="122" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P121">
+        <v>2023.0920000000001</v>
+      </c>
+    </row>
+    <row r="122" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A122" s="1">
         <v>44732</v>
       </c>
@@ -6192,8 +6576,11 @@
       <c r="O122">
         <v>66350.31</v>
       </c>
-    </row>
-    <row r="123" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P122">
+        <v>2023.0920000000001</v>
+      </c>
+    </row>
+    <row r="123" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A123" s="1">
         <v>44733</v>
       </c>
@@ -6239,8 +6626,11 @@
       <c r="O123">
         <v>66747.23</v>
       </c>
-    </row>
-    <row r="124" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P123">
+        <v>2023.0920000000001</v>
+      </c>
+    </row>
+    <row r="124" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A124" s="1">
         <v>44734</v>
       </c>
@@ -6286,8 +6676,11 @@
       <c r="O124">
         <v>65712.679999999993</v>
       </c>
-    </row>
-    <row r="125" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P124">
+        <v>2023.0920000000001</v>
+      </c>
+    </row>
+    <row r="125" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A125" s="1">
         <v>44735</v>
       </c>
@@ -6333,8 +6726,11 @@
       <c r="O125">
         <v>65295.42</v>
       </c>
-    </row>
-    <row r="126" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P125">
+        <v>2023.0920000000001</v>
+      </c>
+    </row>
+    <row r="126" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A126" s="1">
         <v>44736</v>
       </c>
@@ -6380,8 +6776,11 @@
       <c r="O126">
         <v>66348.75</v>
       </c>
-    </row>
-    <row r="127" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P126">
+        <v>2023.0920000000001</v>
+      </c>
+    </row>
+    <row r="127" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A127" s="1">
         <v>44739</v>
       </c>
@@ -6427,8 +6826,11 @@
       <c r="O127">
         <v>67826.78</v>
       </c>
-    </row>
-    <row r="128" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P127">
+        <v>2023.0920000000001</v>
+      </c>
+    </row>
+    <row r="128" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A128" s="1">
         <v>44740</v>
       </c>
@@ -6474,8 +6876,11 @@
       <c r="O128">
         <v>68058.12</v>
       </c>
-    </row>
-    <row r="129" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P128">
+        <v>2023.1220000000001</v>
+      </c>
+    </row>
+    <row r="129" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A129" s="1">
         <v>44741</v>
       </c>
@@ -6521,8 +6926,11 @@
       <c r="O129">
         <v>67747.41</v>
       </c>
-    </row>
-    <row r="130" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P129">
+        <v>2023.1220000000001</v>
+      </c>
+    </row>
+    <row r="130" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A130" s="1">
         <v>44742</v>
       </c>
@@ -6568,8 +6976,11 @@
       <c r="O130">
         <v>66223.31</v>
       </c>
-    </row>
-    <row r="131" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P130">
+        <v>2023.1220000000001</v>
+      </c>
+    </row>
+    <row r="131" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A131" s="1">
         <v>44743</v>
       </c>
@@ -6615,8 +7026,11 @@
       <c r="O131">
         <v>65661.73</v>
       </c>
-    </row>
-    <row r="132" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P131">
+        <v>2023.1220000000001</v>
+      </c>
+    </row>
+    <row r="132" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A132" s="1">
         <v>44746</v>
       </c>
@@ -6662,8 +7076,11 @@
       <c r="O132">
         <v>67024.820000000007</v>
       </c>
-    </row>
-    <row r="133" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P132">
+        <v>2023.1220000000001</v>
+      </c>
+    </row>
+    <row r="133" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A133" s="1">
         <v>44747</v>
       </c>
@@ -6709,8 +7126,11 @@
       <c r="O133">
         <v>65005.81</v>
       </c>
-    </row>
-    <row r="134" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P133">
+        <v>2023.1220000000001</v>
+      </c>
+    </row>
+    <row r="134" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A134" s="1">
         <v>44748</v>
       </c>
@@ -6756,8 +7176,11 @@
       <c r="O134">
         <v>65756.36</v>
       </c>
-    </row>
-    <row r="135" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P134">
+        <v>2023.1220000000001</v>
+      </c>
+    </row>
+    <row r="135" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A135" s="1">
         <v>44749</v>
       </c>
@@ -6803,8 +7226,11 @@
       <c r="O135">
         <v>67909.289999999994</v>
       </c>
-    </row>
-    <row r="136" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P135">
+        <v>2023.1220000000001</v>
+      </c>
+    </row>
+    <row r="136" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A136" s="1">
         <v>44750</v>
       </c>
@@ -6850,8 +7276,11 @@
       <c r="O136">
         <v>68327.399999999994</v>
       </c>
-    </row>
-    <row r="137" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P136">
+        <v>2023.1220000000001</v>
+      </c>
+    </row>
+    <row r="137" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A137" s="1">
         <v>44753</v>
       </c>
@@ -6897,8 +7326,11 @@
       <c r="O137">
         <v>67226.75</v>
       </c>
-    </row>
-    <row r="138" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P137">
+        <v>2023.1220000000001</v>
+      </c>
+    </row>
+    <row r="138" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A138" s="1">
         <v>44754</v>
       </c>
@@ -6944,8 +7376,11 @@
       <c r="O138">
         <v>67163.710000000006</v>
       </c>
-    </row>
-    <row r="139" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P138">
+        <v>2023.1220000000001</v>
+      </c>
+    </row>
+    <row r="139" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A139" s="1">
         <v>44755</v>
       </c>
@@ -6991,8 +7426,11 @@
       <c r="O139">
         <v>66142.69</v>
       </c>
-    </row>
-    <row r="140" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P139">
+        <v>2023.1217999999999</v>
+      </c>
+    </row>
+    <row r="140" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A140" s="1">
         <v>44756</v>
       </c>
@@ -7038,8 +7476,11 @@
       <c r="O140">
         <v>64712.88</v>
       </c>
-    </row>
-    <row r="141" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P140">
+        <v>2024.0309999999999</v>
+      </c>
+    </row>
+    <row r="141" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A141" s="1">
         <v>44757</v>
       </c>
@@ -7085,8 +7526,11 @@
       <c r="O141">
         <v>65088.9</v>
       </c>
-    </row>
-    <row r="142" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P141">
+        <v>2024.0318</v>
+      </c>
+    </row>
+    <row r="142" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A142" s="1">
         <v>44760</v>
       </c>
@@ -7132,8 +7576,11 @@
       <c r="O142">
         <v>67016.14</v>
       </c>
-    </row>
-    <row r="143" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P142">
+        <v>2024.0319999999999</v>
+      </c>
+    </row>
+    <row r="143" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A143" s="1">
         <v>44761</v>
       </c>
@@ -7179,8 +7626,11 @@
       <c r="O143">
         <v>67785.039999999994</v>
       </c>
-    </row>
-    <row r="144" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P143">
+        <v>2024.0319999999999</v>
+      </c>
+    </row>
+    <row r="144" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A144" s="1">
         <v>44762</v>
       </c>
@@ -7226,8 +7676,11 @@
       <c r="O144">
         <v>67652.460000000006</v>
       </c>
-    </row>
-    <row r="145" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P144">
+        <v>2024.0319999999999</v>
+      </c>
+    </row>
+    <row r="145" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A145" s="1">
         <v>44763</v>
       </c>
@@ -7273,8 +7726,11 @@
       <c r="O145">
         <v>67907.240000000005</v>
       </c>
-    </row>
-    <row r="146" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P145">
+        <v>2024.0318</v>
+      </c>
+    </row>
+    <row r="146" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A146" s="1">
         <v>44764</v>
       </c>
@@ -7320,8 +7776,11 @@
       <c r="O146">
         <v>68069.58</v>
       </c>
-    </row>
-    <row r="147" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P146">
+        <v>2024.0319999999999</v>
+      </c>
+    </row>
+    <row r="147" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A147" s="1">
         <v>44767</v>
       </c>
@@ -7367,8 +7826,11 @@
       <c r="O147">
         <v>67749.789999999994</v>
       </c>
-    </row>
-    <row r="148" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P147">
+        <v>2024.0319999999999</v>
+      </c>
+    </row>
+    <row r="148" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A148" s="1">
         <v>44768</v>
       </c>
@@ -7414,8 +7876,11 @@
       <c r="O148">
         <v>68421.8</v>
       </c>
-    </row>
-    <row r="149" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P148">
+        <v>2024.0319999999999</v>
+      </c>
+    </row>
+    <row r="149" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A149" s="1">
         <v>44769</v>
       </c>
@@ -7461,8 +7926,11 @@
       <c r="O149">
         <v>68424.97</v>
       </c>
-    </row>
-    <row r="150" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P149">
+        <v>2024.0319999999999</v>
+      </c>
+    </row>
+    <row r="150" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A150" s="1">
         <v>44770</v>
       </c>
@@ -7508,8 +7976,11 @@
       <c r="O150">
         <v>68610.75</v>
       </c>
-    </row>
-    <row r="151" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P150">
+        <v>2024.0319999999999</v>
+      </c>
+    </row>
+    <row r="151" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A151" s="1">
         <v>44771</v>
       </c>
@@ -7555,8 +8026,11 @@
       <c r="O151">
         <v>68934.009999999995</v>
       </c>
-    </row>
-    <row r="152" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P151">
+        <v>2024.0319999999999</v>
+      </c>
+    </row>
+    <row r="152" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A152" s="1">
         <v>44774</v>
       </c>
@@ -7602,8 +8076,11 @@
       <c r="O152">
         <v>68642.59</v>
       </c>
-    </row>
-    <row r="153" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P152">
+        <v>2024.0319999999999</v>
+      </c>
+    </row>
+    <row r="153" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A153" s="1">
         <v>44775</v>
       </c>
@@ -7649,8 +8126,11 @@
       <c r="O153">
         <v>68002.23</v>
       </c>
-    </row>
-    <row r="154" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P153">
+        <v>2024.0409999999999</v>
+      </c>
+    </row>
+    <row r="154" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A154" s="1">
         <v>44776</v>
       </c>
@@ -7696,8 +8176,11 @@
       <c r="O154">
         <v>68610.570000000007</v>
       </c>
-    </row>
-    <row r="155" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P154">
+        <v>2024.0409999999999</v>
+      </c>
+    </row>
+    <row r="155" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A155" s="1">
         <v>44777</v>
       </c>
@@ -7743,8 +8226,11 @@
       <c r="O155">
         <v>68717.02</v>
       </c>
-    </row>
-    <row r="156" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P155">
+        <v>2024.0619999999999</v>
+      </c>
+    </row>
+    <row r="156" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A156" s="1">
         <v>44778</v>
       </c>
@@ -7790,8 +8276,11 @@
       <c r="O156">
         <v>69519.27</v>
       </c>
-    </row>
-    <row r="157" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P156">
+        <v>2024.0619999999999</v>
+      </c>
+    </row>
+    <row r="157" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A157" s="1">
         <v>44781</v>
       </c>
@@ -7837,8 +8326,11 @@
       <c r="O157">
         <v>70266.13</v>
       </c>
-    </row>
-    <row r="158" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P157">
+        <v>2024.0619999999999</v>
+      </c>
+    </row>
+    <row r="158" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A158" s="1">
         <v>44782</v>
       </c>
@@ -7884,8 +8376,11 @@
       <c r="O158">
         <v>70266.13</v>
       </c>
-    </row>
-    <row r="159" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P158">
+        <v>2024.0619999999999</v>
+      </c>
+    </row>
+    <row r="159" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A159" s="1">
         <v>44783</v>
       </c>
@@ -7931,8 +8426,11 @@
       <c r="O159">
         <v>69744.899999999994</v>
       </c>
-    </row>
-    <row r="160" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P159">
+        <v>2024.0619999999999</v>
+      </c>
+    </row>
+    <row r="160" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A160" s="1">
         <v>44784</v>
       </c>
@@ -7978,8 +8476,11 @@
       <c r="O160">
         <v>71264.77</v>
       </c>
-    </row>
-    <row r="161" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P160">
+        <v>2024.0619999999999</v>
+      </c>
+    </row>
+    <row r="161" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A161" s="1">
         <v>44785</v>
       </c>
@@ -8025,8 +8526,11 @@
       <c r="O161">
         <v>70731.320000000007</v>
       </c>
-    </row>
-    <row r="162" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P161">
+        <v>2024.0619999999999</v>
+      </c>
+    </row>
+    <row r="162" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A162" s="1">
         <v>44788</v>
       </c>
@@ -8072,8 +8576,11 @@
       <c r="O162">
         <v>70740.63</v>
       </c>
-    </row>
-    <row r="163" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P162">
+        <v>2024.0619999999999</v>
+      </c>
+    </row>
+    <row r="163" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A163" s="1">
         <v>44789</v>
       </c>
@@ -8119,8 +8626,11 @@
       <c r="O163">
         <v>71504.69</v>
       </c>
-    </row>
-    <row r="164" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P163">
+        <v>2024.0619999999999</v>
+      </c>
+    </row>
+    <row r="164" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A164" s="1">
         <v>44790</v>
       </c>
@@ -8166,8 +8676,11 @@
       <c r="O164">
         <v>70967.350000000006</v>
       </c>
-    </row>
-    <row r="165" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P164">
+        <v>2024.0619999999999</v>
+      </c>
+    </row>
+    <row r="165" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A165" s="1">
         <v>44791</v>
       </c>
@@ -8213,8 +8726,11 @@
       <c r="O165">
         <v>71011.38</v>
       </c>
-    </row>
-    <row r="166" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P165">
+        <v>2024.07</v>
+      </c>
+    </row>
+    <row r="166" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A166" s="1">
         <v>44792</v>
       </c>
@@ -8260,8 +8776,11 @@
       <c r="O166">
         <v>69719.429999999993</v>
       </c>
-    </row>
-    <row r="167" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P166">
+        <v>2024.07</v>
+      </c>
+    </row>
+    <row r="167" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A167" s="1">
         <v>44795</v>
       </c>
@@ -8308,7 +8827,7 @@
         <v>69195.600000000006</v>
       </c>
     </row>
-    <row r="168" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="168" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A168" s="1">
         <v>44796</v>
       </c>
@@ -8355,7 +8874,7 @@
         <v>69772.27</v>
       </c>
     </row>
-    <row r="169" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="169" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A169" s="1">
         <v>44797</v>
       </c>
@@ -8402,7 +8921,7 @@
         <v>69808.710000000006</v>
       </c>
     </row>
-    <row r="170" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="170" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A170" s="1">
         <v>44798</v>
       </c>
@@ -8449,7 +8968,7 @@
         <v>70340.7</v>
       </c>
     </row>
-    <row r="171" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="171" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A171" s="1">
         <v>44799</v>
       </c>
@@ -8496,7 +9015,7 @@
         <v>70173.09</v>
       </c>
     </row>
-    <row r="172" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="172" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A172" s="1">
         <v>44802</v>
       </c>
@@ -8543,7 +9062,7 @@
         <v>69207.02</v>
       </c>
     </row>
-    <row r="173" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="173" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A173" s="1">
         <v>44803</v>
       </c>
@@ -8590,7 +9109,7 @@
         <v>67900.479999999996</v>
       </c>
     </row>
-    <row r="174" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="174" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A174" s="1">
         <v>44804</v>
       </c>
@@ -8637,7 +9156,7 @@
         <v>67257.14</v>
       </c>
     </row>
-    <row r="175" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="175" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A175" s="1">
         <v>44805</v>
       </c>
@@ -8684,7 +9203,7 @@
         <v>66021.710000000006</v>
       </c>
     </row>
-    <row r="176" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="176" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A176" s="1">
         <v>44806</v>
       </c>
@@ -51640,6 +52159,1367 @@
       </c>
       <c r="O1089">
         <v>121114.3</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6C283D23-5F75-4329-A1F3-1A792FF2A40D}">
+  <dimension ref="A1:B171"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>15</v>
+      </c>
+      <c r="B1" s="1">
+        <v>44564</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B4" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B5" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>0</v>
+      </c>
+      <c r="B6" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A7" s="1">
+        <v>44609</v>
+      </c>
+      <c r="B7">
+        <v>2022.0219999999999</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A8" s="1">
+        <v>44610</v>
+      </c>
+      <c r="B8">
+        <v>2022.0219999999999</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A9" s="1">
+        <v>44613</v>
+      </c>
+      <c r="B9">
+        <v>2022.0219999999999</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A10" s="1">
+        <v>44624</v>
+      </c>
+      <c r="B10">
+        <v>2022.0319999999999</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A11" s="1">
+        <v>44627</v>
+      </c>
+      <c r="B11">
+        <v>2022.0319999999999</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A12" s="1">
+        <v>44628</v>
+      </c>
+      <c r="B12">
+        <v>2022.0319999999999</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A13" s="1">
+        <v>44629</v>
+      </c>
+      <c r="B13">
+        <v>2022.0319999999999</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A14" s="1">
+        <v>44630</v>
+      </c>
+      <c r="B14">
+        <v>2022.0319999999999</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A15" s="1">
+        <v>44631</v>
+      </c>
+      <c r="B15">
+        <v>2022.0319999999999</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A16" s="1">
+        <v>44634</v>
+      </c>
+      <c r="B16">
+        <v>2022.0319999999999</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A17" s="1">
+        <v>44635</v>
+      </c>
+      <c r="B17">
+        <v>2022.0319999999999</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A18" s="1">
+        <v>44636</v>
+      </c>
+      <c r="B18">
+        <v>2022.0319999999999</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A19" s="1">
+        <v>44637</v>
+      </c>
+      <c r="B19">
+        <v>2022.0319999999999</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A20" s="1">
+        <v>44638</v>
+      </c>
+      <c r="B20">
+        <v>2022.0319999999999</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A21" s="1">
+        <v>44641</v>
+      </c>
+      <c r="B21">
+        <v>2022.0319999999999</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A22" s="1">
+        <v>44651</v>
+      </c>
+      <c r="B22">
+        <v>2022.0404000000001</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A23" s="1">
+        <v>44652</v>
+      </c>
+      <c r="B23">
+        <v>2022.04</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A24" s="1">
+        <v>44655</v>
+      </c>
+      <c r="B24">
+        <v>2022.04</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A25" s="1">
+        <v>44677</v>
+      </c>
+      <c r="B25">
+        <v>2022.0429999999999</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A26" s="1">
+        <v>44678</v>
+      </c>
+      <c r="B26">
+        <v>2022.0429999999999</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A27" s="1">
+        <v>44679</v>
+      </c>
+      <c r="B27">
+        <v>2022.05</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A28" s="1">
+        <v>44680</v>
+      </c>
+      <c r="B28">
+        <v>2022.05</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A29" s="1">
+        <v>44683</v>
+      </c>
+      <c r="B29">
+        <v>2022.0501999999999</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A30" s="1">
+        <v>44715</v>
+      </c>
+      <c r="B30">
+        <v>2022.0619999999999</v>
+      </c>
+    </row>
+    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A31" s="1">
+        <v>44719</v>
+      </c>
+      <c r="B31">
+        <v>2022.0619999999999</v>
+      </c>
+    </row>
+    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A32" s="1">
+        <v>44720</v>
+      </c>
+      <c r="B32">
+        <v>2022.0619999999999</v>
+      </c>
+    </row>
+    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A33" s="1">
+        <v>44721</v>
+      </c>
+      <c r="B33">
+        <v>2022.0619999999999</v>
+      </c>
+    </row>
+    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A34" s="1">
+        <v>44722</v>
+      </c>
+      <c r="B34">
+        <v>2022.0619999999999</v>
+      </c>
+    </row>
+    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A35" s="1">
+        <v>44725</v>
+      </c>
+      <c r="B35">
+        <v>2022.0619999999999</v>
+      </c>
+    </row>
+    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A36" s="1">
+        <v>44726</v>
+      </c>
+      <c r="B36">
+        <v>2022.0619999999999</v>
+      </c>
+    </row>
+    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A37" s="1">
+        <v>44727</v>
+      </c>
+      <c r="B37">
+        <v>2022.0619999999999</v>
+      </c>
+    </row>
+    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A38" s="1">
+        <v>44728</v>
+      </c>
+      <c r="B38">
+        <v>2022.0619999999999</v>
+      </c>
+    </row>
+    <row r="39" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A39" s="1">
+        <v>44729</v>
+      </c>
+      <c r="B39">
+        <v>2022.0619999999999</v>
+      </c>
+    </row>
+    <row r="40" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A40" s="1">
+        <v>44732</v>
+      </c>
+      <c r="B40">
+        <v>2022.0619999999999</v>
+      </c>
+    </row>
+    <row r="41" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A41" s="1">
+        <v>44761</v>
+      </c>
+      <c r="B41">
+        <v>2022.0721000000001</v>
+      </c>
+    </row>
+    <row r="42" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A42" s="1">
+        <v>44762</v>
+      </c>
+      <c r="B42">
+        <v>2022.0719999999999</v>
+      </c>
+    </row>
+    <row r="43" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A43" s="1">
+        <v>44763</v>
+      </c>
+      <c r="B43">
+        <v>2022.0719999999999</v>
+      </c>
+    </row>
+    <row r="44" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A44" s="1">
+        <v>44806</v>
+      </c>
+      <c r="B44">
+        <v>2022.0920000000001</v>
+      </c>
+    </row>
+    <row r="45" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A45" s="1">
+        <v>44809</v>
+      </c>
+      <c r="B45">
+        <v>2022.0920000000001</v>
+      </c>
+    </row>
+    <row r="46" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A46" s="1">
+        <v>44810</v>
+      </c>
+      <c r="B46">
+        <v>2022.0920000000001</v>
+      </c>
+    </row>
+    <row r="47" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A47" s="1">
+        <v>44811</v>
+      </c>
+      <c r="B47">
+        <v>2022.0920000000001</v>
+      </c>
+    </row>
+    <row r="48" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A48" s="1">
+        <v>44812</v>
+      </c>
+      <c r="B48">
+        <v>2022.0920000000001</v>
+      </c>
+    </row>
+    <row r="49" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A49" s="1">
+        <v>44813</v>
+      </c>
+      <c r="B49">
+        <v>2022.0920000000001</v>
+      </c>
+    </row>
+    <row r="50" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A50" s="1">
+        <v>44816</v>
+      </c>
+      <c r="B50">
+        <v>2022.0920000000001</v>
+      </c>
+    </row>
+    <row r="51" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A51" s="1">
+        <v>44817</v>
+      </c>
+      <c r="B51">
+        <v>2022.0920000000001</v>
+      </c>
+    </row>
+    <row r="52" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A52" s="1">
+        <v>44818</v>
+      </c>
+      <c r="B52">
+        <v>2022.0920000000001</v>
+      </c>
+    </row>
+    <row r="53" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A53" s="1">
+        <v>44819</v>
+      </c>
+      <c r="B53">
+        <v>2022.0920000000001</v>
+      </c>
+    </row>
+    <row r="54" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A54" s="1">
+        <v>44820</v>
+      </c>
+      <c r="B54">
+        <v>2022.0920000000001</v>
+      </c>
+    </row>
+    <row r="55" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A55" s="1">
+        <v>44823</v>
+      </c>
+      <c r="B55">
+        <v>2022.0920000000001</v>
+      </c>
+    </row>
+    <row r="56" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A56" s="1">
+        <v>44824</v>
+      </c>
+      <c r="B56">
+        <v>2022.0930000000001</v>
+      </c>
+    </row>
+    <row r="57" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A57" s="1">
+        <v>44825</v>
+      </c>
+      <c r="B57">
+        <v>2022.0930000000001</v>
+      </c>
+    </row>
+    <row r="58" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A58" s="1">
+        <v>44826</v>
+      </c>
+      <c r="B58">
+        <v>2022.0930000000001</v>
+      </c>
+    </row>
+    <row r="59" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A59" s="1">
+        <v>44827</v>
+      </c>
+      <c r="B59">
+        <v>2022.0930000000001</v>
+      </c>
+    </row>
+    <row r="60" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A60" s="1">
+        <v>44831</v>
+      </c>
+      <c r="B60">
+        <v>2022.0930000000001</v>
+      </c>
+    </row>
+    <row r="61" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A61" s="1">
+        <v>44876</v>
+      </c>
+      <c r="B61">
+        <v>2022.1122</v>
+      </c>
+    </row>
+    <row r="62" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A62" s="1">
+        <v>44879</v>
+      </c>
+      <c r="B62">
+        <v>2022.1120000000001</v>
+      </c>
+    </row>
+    <row r="63" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A63" s="1">
+        <v>44880</v>
+      </c>
+      <c r="B63">
+        <v>2022.1120000000001</v>
+      </c>
+    </row>
+    <row r="64" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A64" s="1">
+        <v>44881</v>
+      </c>
+      <c r="B64">
+        <v>2022.1122</v>
+      </c>
+    </row>
+    <row r="65" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A65" s="1">
+        <v>44882</v>
+      </c>
+      <c r="B65">
+        <v>2022.1122</v>
+      </c>
+    </row>
+    <row r="66" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A66" s="1">
+        <v>44883</v>
+      </c>
+      <c r="B66">
+        <v>2022.1120000000001</v>
+      </c>
+    </row>
+    <row r="67" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A67" s="1">
+        <v>44886</v>
+      </c>
+      <c r="B67">
+        <v>2022.1120000000001</v>
+      </c>
+    </row>
+    <row r="68" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A68" s="1">
+        <v>44887</v>
+      </c>
+      <c r="B68">
+        <v>2022.1120000000001</v>
+      </c>
+    </row>
+    <row r="69" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A69" s="1">
+        <v>44897</v>
+      </c>
+      <c r="B69">
+        <v>2022.1220000000001</v>
+      </c>
+    </row>
+    <row r="70" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A70" s="1">
+        <v>44900</v>
+      </c>
+      <c r="B70">
+        <v>2022.1220000000001</v>
+      </c>
+    </row>
+    <row r="71" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A71" s="1">
+        <v>44901</v>
+      </c>
+      <c r="B71">
+        <v>2022.1220000000001</v>
+      </c>
+    </row>
+    <row r="72" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A72" s="1">
+        <v>44902</v>
+      </c>
+      <c r="B72">
+        <v>2022.1220000000001</v>
+      </c>
+    </row>
+    <row r="73" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A73" s="1">
+        <v>44903</v>
+      </c>
+      <c r="B73">
+        <v>2022.1220000000001</v>
+      </c>
+    </row>
+    <row r="74" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A74" s="1">
+        <v>44904</v>
+      </c>
+      <c r="B74">
+        <v>2022.1220000000001</v>
+      </c>
+    </row>
+    <row r="75" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A75" s="1">
+        <v>44907</v>
+      </c>
+      <c r="B75">
+        <v>2022.1220000000001</v>
+      </c>
+    </row>
+    <row r="76" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A76" s="1">
+        <v>44908</v>
+      </c>
+      <c r="B76">
+        <v>2022.1220000000001</v>
+      </c>
+    </row>
+    <row r="77" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A77" s="1">
+        <v>44909</v>
+      </c>
+      <c r="B77">
+        <v>2022.1220000000001</v>
+      </c>
+    </row>
+    <row r="78" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A78" s="1">
+        <v>44910</v>
+      </c>
+      <c r="B78">
+        <v>2022.1219000000001</v>
+      </c>
+    </row>
+    <row r="79" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A79" s="1">
+        <v>44911</v>
+      </c>
+      <c r="B79">
+        <v>2022.1220000000001</v>
+      </c>
+    </row>
+    <row r="80" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A80" s="1">
+        <v>44914</v>
+      </c>
+      <c r="B80">
+        <v>2022.1220000000001</v>
+      </c>
+    </row>
+    <row r="81" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A81" s="1">
+        <v>44972</v>
+      </c>
+      <c r="B81">
+        <v>2023.0219999999999</v>
+      </c>
+    </row>
+    <row r="82" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A82" s="1">
+        <v>44973</v>
+      </c>
+      <c r="B82">
+        <v>2023.0219999999999</v>
+      </c>
+    </row>
+    <row r="83" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A83" s="1">
+        <v>44974</v>
+      </c>
+      <c r="B83">
+        <v>2023.0219999999999</v>
+      </c>
+    </row>
+    <row r="84" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A84" s="1">
+        <v>44977</v>
+      </c>
+      <c r="B84">
+        <v>2023.0219999999999</v>
+      </c>
+    </row>
+    <row r="85" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A85" s="1">
+        <v>44988</v>
+      </c>
+      <c r="B85">
+        <v>2023.0319999999999</v>
+      </c>
+    </row>
+    <row r="86" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A86" s="1">
+        <v>44991</v>
+      </c>
+      <c r="B86">
+        <v>2023.0319999999999</v>
+      </c>
+    </row>
+    <row r="87" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A87" s="1">
+        <v>44992</v>
+      </c>
+      <c r="B87">
+        <v>2023.0319999999999</v>
+      </c>
+    </row>
+    <row r="88" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A88" s="1">
+        <v>44993</v>
+      </c>
+      <c r="B88">
+        <v>2023.0319999999999</v>
+      </c>
+    </row>
+    <row r="89" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A89" s="1">
+        <v>44994</v>
+      </c>
+      <c r="B89">
+        <v>2023.0319999999999</v>
+      </c>
+    </row>
+    <row r="90" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A90" s="1">
+        <v>44995</v>
+      </c>
+      <c r="B90">
+        <v>2023.0319999999999</v>
+      </c>
+    </row>
+    <row r="91" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A91" s="1">
+        <v>44998</v>
+      </c>
+      <c r="B91">
+        <v>2023.0319999999999</v>
+      </c>
+    </row>
+    <row r="92" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A92" s="1">
+        <v>44999</v>
+      </c>
+      <c r="B92">
+        <v>2023.0319999999999</v>
+      </c>
+    </row>
+    <row r="93" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A93" s="1">
+        <v>45000</v>
+      </c>
+      <c r="B93">
+        <v>2023.0319999999999</v>
+      </c>
+    </row>
+    <row r="94" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A94" s="1">
+        <v>45001</v>
+      </c>
+      <c r="B94">
+        <v>2023.0319999999999</v>
+      </c>
+    </row>
+    <row r="95" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A95" s="1">
+        <v>45002</v>
+      </c>
+      <c r="B95">
+        <v>2023.0219999999999</v>
+      </c>
+    </row>
+    <row r="96" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A96" s="1">
+        <v>45005</v>
+      </c>
+      <c r="B96">
+        <v>2023.0319999999999</v>
+      </c>
+    </row>
+    <row r="97" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A97" s="1">
+        <v>45049</v>
+      </c>
+      <c r="B97">
+        <v>2023.0509999999999</v>
+      </c>
+    </row>
+    <row r="98" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A98" s="1">
+        <v>45050</v>
+      </c>
+      <c r="B98">
+        <v>2023.0509999999999</v>
+      </c>
+    </row>
+    <row r="99" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A99" s="1">
+        <v>45051</v>
+      </c>
+      <c r="B99">
+        <v>2023.0509999999999</v>
+      </c>
+    </row>
+    <row r="100" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A100" s="1">
+        <v>45054</v>
+      </c>
+      <c r="B100">
+        <v>2023.0509999999999</v>
+      </c>
+    </row>
+    <row r="101" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A101" s="1">
+        <v>45055</v>
+      </c>
+      <c r="B101">
+        <v>2023.0509999999999</v>
+      </c>
+    </row>
+    <row r="102" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A102" s="1">
+        <v>45056</v>
+      </c>
+      <c r="B102">
+        <v>2023.0509999999999</v>
+      </c>
+    </row>
+    <row r="103" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A103" s="1">
+        <v>45057</v>
+      </c>
+      <c r="B103">
+        <v>2023.0509999999999</v>
+      </c>
+    </row>
+    <row r="104" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A104" s="1">
+        <v>45079</v>
+      </c>
+      <c r="B104">
+        <v>2023.0619999999999</v>
+      </c>
+    </row>
+    <row r="105" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A105" s="1">
+        <v>45083</v>
+      </c>
+      <c r="B105">
+        <v>2023.0619999999999</v>
+      </c>
+    </row>
+    <row r="106" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A106" s="1">
+        <v>45084</v>
+      </c>
+      <c r="B106">
+        <v>2023.0619999999999</v>
+      </c>
+    </row>
+    <row r="107" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A107" s="1">
+        <v>45085</v>
+      </c>
+      <c r="B107">
+        <v>2023.0619999999999</v>
+      </c>
+    </row>
+    <row r="108" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A108" s="1">
+        <v>45086</v>
+      </c>
+      <c r="B108">
+        <v>2023.0619999999999</v>
+      </c>
+    </row>
+    <row r="109" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A109" s="1">
+        <v>45089</v>
+      </c>
+      <c r="B109">
+        <v>2023.0619999999999</v>
+      </c>
+    </row>
+    <row r="110" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A110" s="1">
+        <v>45090</v>
+      </c>
+      <c r="B110">
+        <v>2023.0619999999999</v>
+      </c>
+    </row>
+    <row r="111" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A111" s="1">
+        <v>45091</v>
+      </c>
+      <c r="B111">
+        <v>2023.0619999999999</v>
+      </c>
+    </row>
+    <row r="112" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A112" s="1">
+        <v>45092</v>
+      </c>
+      <c r="B112">
+        <v>2023.0619999999999</v>
+      </c>
+    </row>
+    <row r="113" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A113" s="1">
+        <v>45093</v>
+      </c>
+      <c r="B113">
+        <v>2023.0619999999999</v>
+      </c>
+    </row>
+    <row r="114" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A114" s="1">
+        <v>45096</v>
+      </c>
+      <c r="B114">
+        <v>2023.0626</v>
+      </c>
+    </row>
+    <row r="115" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A115" s="1">
+        <v>45097</v>
+      </c>
+      <c r="B115">
+        <v>2023.0626</v>
+      </c>
+    </row>
+    <row r="116" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A116" s="1">
+        <v>45098</v>
+      </c>
+      <c r="B116">
+        <v>2023.0630000000001</v>
+      </c>
+    </row>
+    <row r="117" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A117" s="1">
+        <v>45099</v>
+      </c>
+      <c r="B117">
+        <v>2023.0630000000001</v>
+      </c>
+    </row>
+    <row r="118" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A118" s="1">
+        <v>45100</v>
+      </c>
+      <c r="B118">
+        <v>2023.0630000000001</v>
+      </c>
+    </row>
+    <row r="119" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A119" s="1">
+        <v>45103</v>
+      </c>
+      <c r="B119">
+        <v>2023.0630000000001</v>
+      </c>
+    </row>
+    <row r="120" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A120" s="1">
+        <v>45107</v>
+      </c>
+      <c r="B120">
+        <v>2023.0709999999999</v>
+      </c>
+    </row>
+    <row r="121" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A121" s="1">
+        <v>45170</v>
+      </c>
+      <c r="B121">
+        <v>2023.0920000000001</v>
+      </c>
+    </row>
+    <row r="122" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A122" s="1">
+        <v>45173</v>
+      </c>
+      <c r="B122">
+        <v>2023.0920000000001</v>
+      </c>
+    </row>
+    <row r="123" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A123" s="1">
+        <v>45174</v>
+      </c>
+      <c r="B123">
+        <v>2023.0920000000001</v>
+      </c>
+    </row>
+    <row r="124" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A124" s="1">
+        <v>45175</v>
+      </c>
+      <c r="B124">
+        <v>2023.0920000000001</v>
+      </c>
+    </row>
+    <row r="125" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A125" s="1">
+        <v>45176</v>
+      </c>
+      <c r="B125">
+        <v>2023.0920000000001</v>
+      </c>
+    </row>
+    <row r="126" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A126" s="1">
+        <v>45177</v>
+      </c>
+      <c r="B126">
+        <v>2023.0920000000001</v>
+      </c>
+    </row>
+    <row r="127" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A127" s="1">
+        <v>45180</v>
+      </c>
+      <c r="B127">
+        <v>2023.0920000000001</v>
+      </c>
+    </row>
+    <row r="128" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A128" s="1">
+        <v>45181</v>
+      </c>
+      <c r="B128">
+        <v>2023.0920000000001</v>
+      </c>
+    </row>
+    <row r="129" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A129" s="1">
+        <v>45182</v>
+      </c>
+      <c r="B129">
+        <v>2023.0920000000001</v>
+      </c>
+    </row>
+    <row r="130" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A130" s="1">
+        <v>45183</v>
+      </c>
+      <c r="B130">
+        <v>2023.0920000000001</v>
+      </c>
+    </row>
+    <row r="131" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A131" s="1">
+        <v>45184</v>
+      </c>
+      <c r="B131">
+        <v>2023.0920000000001</v>
+      </c>
+    </row>
+    <row r="132" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A132" s="1">
+        <v>45187</v>
+      </c>
+      <c r="B132">
+        <v>2023.0920000000001</v>
+      </c>
+    </row>
+    <row r="133" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A133" s="1">
+        <v>45261</v>
+      </c>
+      <c r="B133">
+        <v>2023.1220000000001</v>
+      </c>
+    </row>
+    <row r="134" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A134" s="1">
+        <v>45264</v>
+      </c>
+      <c r="B134">
+        <v>2023.1220000000001</v>
+      </c>
+    </row>
+    <row r="135" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A135" s="1">
+        <v>45265</v>
+      </c>
+      <c r="B135">
+        <v>2023.1220000000001</v>
+      </c>
+    </row>
+    <row r="136" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A136" s="1">
+        <v>45266</v>
+      </c>
+      <c r="B136">
+        <v>2023.1220000000001</v>
+      </c>
+    </row>
+    <row r="137" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A137" s="1">
+        <v>45267</v>
+      </c>
+      <c r="B137">
+        <v>2023.1220000000001</v>
+      </c>
+    </row>
+    <row r="138" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A138" s="1">
+        <v>45268</v>
+      </c>
+      <c r="B138">
+        <v>2023.1220000000001</v>
+      </c>
+    </row>
+    <row r="139" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A139" s="1">
+        <v>45271</v>
+      </c>
+      <c r="B139">
+        <v>2023.1220000000001</v>
+      </c>
+    </row>
+    <row r="140" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A140" s="1">
+        <v>45272</v>
+      </c>
+      <c r="B140">
+        <v>2023.1220000000001</v>
+      </c>
+    </row>
+    <row r="141" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A141" s="1">
+        <v>45273</v>
+      </c>
+      <c r="B141">
+        <v>2023.1220000000001</v>
+      </c>
+    </row>
+    <row r="142" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A142" s="1">
+        <v>45274</v>
+      </c>
+      <c r="B142">
+        <v>2023.1220000000001</v>
+      </c>
+    </row>
+    <row r="143" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A143" s="1">
+        <v>45275</v>
+      </c>
+      <c r="B143">
+        <v>2023.1220000000001</v>
+      </c>
+    </row>
+    <row r="144" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A144" s="1">
+        <v>45278</v>
+      </c>
+      <c r="B144">
+        <v>2023.1217999999999</v>
+      </c>
+    </row>
+    <row r="145" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A145" s="1">
+        <v>45351</v>
+      </c>
+      <c r="B145">
+        <v>2024.0309999999999</v>
+      </c>
+    </row>
+    <row r="146" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A146" s="1">
+        <v>45352</v>
+      </c>
+      <c r="B146">
+        <v>2024.0318</v>
+      </c>
+    </row>
+    <row r="147" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A147" s="1">
+        <v>45355</v>
+      </c>
+      <c r="B147">
+        <v>2024.0319999999999</v>
+      </c>
+    </row>
+    <row r="148" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A148" s="1">
+        <v>45356</v>
+      </c>
+      <c r="B148">
+        <v>2024.0319999999999</v>
+      </c>
+    </row>
+    <row r="149" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A149" s="1">
+        <v>45357</v>
+      </c>
+      <c r="B149">
+        <v>2024.0319999999999</v>
+      </c>
+    </row>
+    <row r="150" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A150" s="1">
+        <v>45358</v>
+      </c>
+      <c r="B150">
+        <v>2024.0318</v>
+      </c>
+    </row>
+    <row r="151" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A151" s="1">
+        <v>45359</v>
+      </c>
+      <c r="B151">
+        <v>2024.0319999999999</v>
+      </c>
+    </row>
+    <row r="152" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A152" s="1">
+        <v>45362</v>
+      </c>
+      <c r="B152">
+        <v>2024.0319999999999</v>
+      </c>
+    </row>
+    <row r="153" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A153" s="1">
+        <v>45363</v>
+      </c>
+      <c r="B153">
+        <v>2024.0319999999999</v>
+      </c>
+    </row>
+    <row r="154" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A154" s="1">
+        <v>45364</v>
+      </c>
+      <c r="B154">
+        <v>2024.0319999999999</v>
+      </c>
+    </row>
+    <row r="155" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A155" s="1">
+        <v>45365</v>
+      </c>
+      <c r="B155">
+        <v>2024.0319999999999</v>
+      </c>
+    </row>
+    <row r="156" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A156" s="1">
+        <v>45366</v>
+      </c>
+      <c r="B156">
+        <v>2024.0319999999999</v>
+      </c>
+    </row>
+    <row r="157" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A157" s="1">
+        <v>45369</v>
+      </c>
+      <c r="B157">
+        <v>2024.0319999999999</v>
+      </c>
+    </row>
+    <row r="158" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A158" s="1">
+        <v>45390</v>
+      </c>
+      <c r="B158">
+        <v>2024.0409999999999</v>
+      </c>
+    </row>
+    <row r="159" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A159" s="1">
+        <v>45391</v>
+      </c>
+      <c r="B159">
+        <v>2024.0409999999999</v>
+      </c>
+    </row>
+    <row r="160" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A160" s="1">
+        <v>45450</v>
+      </c>
+      <c r="B160">
+        <v>2024.0619999999999</v>
+      </c>
+    </row>
+    <row r="161" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A161" s="1">
+        <v>45453</v>
+      </c>
+      <c r="B161">
+        <v>2024.0619999999999</v>
+      </c>
+    </row>
+    <row r="162" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A162" s="1">
+        <v>45454</v>
+      </c>
+      <c r="B162">
+        <v>2024.0619999999999</v>
+      </c>
+    </row>
+    <row r="163" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A163" s="1">
+        <v>45455</v>
+      </c>
+      <c r="B163">
+        <v>2024.0619999999999</v>
+      </c>
+    </row>
+    <row r="164" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A164" s="1">
+        <v>45456</v>
+      </c>
+      <c r="B164">
+        <v>2024.0619999999999</v>
+      </c>
+    </row>
+    <row r="165" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A165" s="1">
+        <v>45457</v>
+      </c>
+      <c r="B165">
+        <v>2024.0619999999999</v>
+      </c>
+    </row>
+    <row r="166" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A166" s="1">
+        <v>45460</v>
+      </c>
+      <c r="B166">
+        <v>2024.0619999999999</v>
+      </c>
+    </row>
+    <row r="167" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A167" s="1">
+        <v>45461</v>
+      </c>
+      <c r="B167">
+        <v>2024.0619999999999</v>
+      </c>
+    </row>
+    <row r="168" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A168" s="1">
+        <v>45462</v>
+      </c>
+      <c r="B168">
+        <v>2024.0619999999999</v>
+      </c>
+    </row>
+    <row r="169" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A169" s="1">
+        <v>45463</v>
+      </c>
+      <c r="B169">
+        <v>2024.0619999999999</v>
+      </c>
+    </row>
+    <row r="170" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A170" s="1">
+        <v>45464</v>
+      </c>
+      <c r="B170">
+        <v>2024.07</v>
+      </c>
+    </row>
+    <row r="171" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A171" s="1">
+        <v>45467</v>
+      </c>
+      <c r="B171">
+        <v>2024.07</v>
       </c>
     </row>
   </sheetData>
@@ -51648,6 +53528,12 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100EF915A43B80B564FB5795C8E88017F14" ma:contentTypeVersion="4" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="8ed44c28e7bb9d7f9e01620cb3466ad6">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="eac73721-e757-4f17-954f-1a93e8307f3e" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="6517c1d2b64b088cbf7dd5900ecc80da" ns3:_="">
     <xsd:import namespace="eac73721-e757-4f17-954f-1a93e8307f3e"/>
@@ -51791,7 +53677,7 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
@@ -51800,13 +53686,23 @@
 </FormTemplates>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B4C61B63-9C6B-4A17-837D-BBAB8022D1D5}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="eac73721-e757-4f17-954f-1a93e8307f3e"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B824AE4B-9B6A-4FA0-A421-FBE4B2ED7DCE}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -51824,26 +53720,10 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{46BBCC01-D381-4B6C-ABAB-65D23FF8C424}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B4C61B63-9C6B-4A17-837D-BBAB8022D1D5}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="eac73721-e757-4f17-954f-1a93e8307f3e"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>